<commit_message>
Adjusting the data so were sometimes below the minimum threshold
</commit_message>
<xml_diff>
--- a/app/data/bi_diagramm_data.xlsx
+++ b/app/data/bi_diagramm_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeremystieger/Documents/5. Semester/Data analysis with Python/Data FP - JBNS/final-project-jbns/app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B403A3A5-77A0-7B43-ACEC-8326D5BC5AD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{751B1E43-F2E9-E542-82E5-D712590DFF94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="28800" windowHeight="18000" xr2:uid="{3BB1FB84-8839-FB4A-82DC-2EADBF823784}"/>
   </bookViews>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="D7">
         <f t="shared" si="1"/>
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="E7">
         <v>27</v>
@@ -1185,10 +1185,10 @@
         <v>26</v>
       </c>
       <c r="G7">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="H7">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I7">
         <v>30</v>
@@ -1218,7 +1218,7 @@
         <v>25</v>
       </c>
       <c r="R7">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="S7">
         <v>22</v>
@@ -1233,22 +1233,22 @@
         <v>22</v>
       </c>
       <c r="W7">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="X7">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="Y7">
         <v>15</v>
       </c>
       <c r="Z7">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="AA7">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AB7">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="AC7">
         <v>22</v>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="D9">
         <f t="shared" si="1"/>
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="E9">
         <v>28</v>
@@ -1389,7 +1389,7 @@
         <v>22</v>
       </c>
       <c r="G9">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="H9">
         <v>23</v>
@@ -1419,10 +1419,10 @@
         <v>30</v>
       </c>
       <c r="Q9">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="R9">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="S9">
         <v>23</v>
@@ -1434,7 +1434,7 @@
         <v>22</v>
       </c>
       <c r="V9">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="W9">
         <v>22</v>
@@ -1449,13 +1449,13 @@
         <v>29</v>
       </c>
       <c r="AA9">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="AB9">
         <v>23</v>
       </c>
       <c r="AC9">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="AD9">
         <v>357</v>
@@ -1900,7 +1900,7 @@
         <v>25</v>
       </c>
       <c r="G14">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H14">
         <v>43</v>
@@ -1957,7 +1957,7 @@
         <v>22</v>
       </c>
       <c r="Z14">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="AA14">
         <v>107</v>

</xml_diff>

<commit_message>
ridying up the whole webapp and make everythin clean
</commit_message>
<xml_diff>
--- a/app/data/bi_diagramm_data.xlsx
+++ b/app/data/bi_diagramm_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeremystieger/Documents/5. Semester/Data analysis with Python/Data FP - JBNS/final-project-jbns/app/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jelenanaf/Desktop/final-project-jbns/app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{751B1E43-F2E9-E542-82E5-D712590DFF94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CA90E11-9137-7243-B4A4-25D33DE71A5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="28800" windowHeight="18000" xr2:uid="{3BB1FB84-8839-FB4A-82DC-2EADBF823784}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16360" xr2:uid="{3BB1FB84-8839-FB4A-82DC-2EADBF823784}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>

</xml_diff>